<commit_message>
Update LondonCentral address details
</commit_message>
<xml_diff>
--- a/src/main/resources/venueAddressValues.xlsx
+++ b/src/main/resources/venueAddressValues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mehmet.dede/dev/IntelliJ/ecm/ethos-repl-docmosis-service/src/main/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harpreet.jhita/IdeaProjects/ethos-repl-docmosis-service/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681B2C2F-F0E5-BB4E-9120-4737755600F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7A1B35-A7E0-BF4A-AED2-B368436B374C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="9" xr2:uid="{57ECFE3E-99BE-FC40-B6CA-F6152164B97B}"/>
+    <workbookView xWindow="28620" yWindow="-31780" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{57ECFE3E-99BE-FC40-B6CA-F6152164B97B}"/>
   </bookViews>
   <sheets>
     <sheet name="Bristol" sheetId="3" r:id="rId1"/>
@@ -632,9 +632,6 @@
     <t>1st Floor, Ashford House, County Square Shopping Centre, Ashford, TN23 1YB</t>
   </si>
   <si>
-    <t>Victory House, 30-34 Kingsway, London, WC2B 6EX</t>
-  </si>
-  <si>
     <t>London (Central), 4th Floor Fox Court, 30 Brooke Street, London, EC1N 7RS</t>
   </si>
   <si>
@@ -1346,6 +1343,9 @@
   </si>
   <si>
     <t>Glasgow Tribunal Centre, 3 Atlantic Quay, 20 York Street, Glasgow, G2 8GT</t>
+  </si>
+  <si>
+    <t>7 Newgate Street, London, EC1A 7AZ</t>
   </si>
 </sst>
 </file>
@@ -2142,18 +2142,18 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>231</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2174,10 +2174,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2190,138 +2190,138 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>254</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>247</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>237</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>249</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>243</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>245</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -2363,7 +2363,7 @@
         <v>104</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2379,7 +2379,7 @@
         <v>106</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2411,7 +2411,7 @@
         <v>110</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2427,7 +2427,7 @@
         <v>112</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2435,7 +2435,7 @@
         <v>113</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2459,7 +2459,7 @@
         <v>116</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -2491,7 +2491,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2579,7 +2579,7 @@
         <v>131</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -2635,7 +2635,7 @@
         <v>138</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -2651,7 +2651,7 @@
         <v>140</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -2683,7 +2683,7 @@
         <v>144</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -2723,7 +2723,7 @@
         <v>149</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -2739,7 +2739,7 @@
         <v>151</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -2747,7 +2747,7 @@
         <v>152</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -2755,7 +2755,7 @@
         <v>153</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -2795,7 +2795,7 @@
         <v>158</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -2811,7 +2811,7 @@
         <v>160</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -2843,7 +2843,7 @@
         <v>164</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -2851,7 +2851,7 @@
         <v>165</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -2867,7 +2867,7 @@
         <v>167</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -2880,10 +2880,10 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2915,7 +2915,7 @@
         <v>169</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2923,7 +2923,7 @@
         <v>170</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2931,7 +2931,7 @@
         <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2947,7 +2947,7 @@
         <v>89</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2955,7 +2955,7 @@
         <v>90</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2963,7 +2963,7 @@
         <v>172</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2987,7 +2987,7 @@
         <v>174</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2995,7 +2995,7 @@
         <v>175</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3011,15 +3011,15 @@
         <v>177</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>228</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3071,10 +3071,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3111,10 +3111,10 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3153,7 +3153,7 @@
         <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3161,15 +3161,15 @@
         <v>51</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>296</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3216,7 +3216,7 @@
         <v>54</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3310,7 +3310,7 @@
         <v>60</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3318,7 +3318,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3334,7 +3334,7 @@
         <v>63</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3342,7 +3342,7 @@
         <v>64</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3382,7 +3382,7 @@
         <v>69</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3390,7 +3390,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3398,7 +3398,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3427,10 +3427,10 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -3469,7 +3469,7 @@
         <v>75</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3493,7 +3493,7 @@
         <v>78</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3501,7 +3501,7 @@
         <v>79</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3525,7 +3525,7 @@
         <v>81</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3604,7 +3604,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3641,10 +3641,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3660,7 +3660,7 @@
         <v>93</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3668,7 +3668,7 @@
         <v>94</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3739,7 +3739,7 @@
         <v>100</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3747,7 +3747,7 @@
         <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3768,18 +3768,18 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -3788,18 +3788,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4020,18 +4020,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E254D28-D3D4-49BF-9139-FF4FDEF467DC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E21D230-F0FF-46F1-8C9B-DF853E5491B6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E21D230-F0FF-46F1-8C9B-DF853E5491B6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E254D28-D3D4-49BF-9139-FF4FDEF467DC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
RET-6184 & RET-6188 (#2693)
* Update London Central address details in defaults.yml and related tests

* Update telephone number for Bristol tribunal correspondence in defaults.yml and related test

* Update LondonCentral address details

* Update LondonCentral address details
</commit_message>
<xml_diff>
--- a/src/main/resources/venueAddressValues.xlsx
+++ b/src/main/resources/venueAddressValues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mehmet.dede/dev/IntelliJ/ecm/ethos-repl-docmosis-service/src/main/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harpreet.jhita/IdeaProjects/ethos-repl-docmosis-service/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681B2C2F-F0E5-BB4E-9120-4737755600F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021525C4-36F6-5343-945C-45FE108B32DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="9" xr2:uid="{57ECFE3E-99BE-FC40-B6CA-F6152164B97B}"/>
+    <workbookView xWindow="5280" yWindow="1900" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{57ECFE3E-99BE-FC40-B6CA-F6152164B97B}"/>
   </bookViews>
   <sheets>
     <sheet name="Bristol" sheetId="3" r:id="rId1"/>
@@ -632,720 +632,720 @@
     <t>1st Floor, Ashford House, County Square Shopping Centre, Ashford, TN23 1YB</t>
   </si>
   <si>
+    <t>London (Central), 4th Floor Fox Court, 30 Brooke Street, London, EC1N 7RS</t>
+  </si>
+  <si>
+    <t>East London Tribunals, 2nd Floor Import Building, 2 Clove Crescent, London,E 14 2BE</t>
+  </si>
+  <si>
+    <t>Newcastle CFCTC, Barras Bridge, Newcastle upon Tyne, Tyne &amp; Wear, NE1 8QF</t>
+  </si>
+  <si>
+    <t>Victoria Square, Middlesbrough, TS1 2AS</t>
+  </si>
+  <si>
+    <t>Earl Grey Way, North Shields, NE29 6AR</t>
+  </si>
+  <si>
+    <t>North Shields</t>
+  </si>
+  <si>
+    <t>Manchester Employment Tribunals, Alexandra House, 14-22 The Parsonage, Manchester, M3 2JA</t>
+  </si>
+  <si>
+    <t>Employment Tribunals, Third Floor, Civil &amp; Family Court, 35 Vernon Street, Liverpool, L2 2BX</t>
+  </si>
+  <si>
+    <t>Carlisle Combined Court, Courts of Justice, Earl Street, Carlisle, Cumbria, CA1 1DJ</t>
+  </si>
+  <si>
+    <t>Carlisle Magistrates Court, The Court House, Rickergate, Carlisle, CA3 8 QH</t>
+  </si>
+  <si>
+    <t>Barrow Magistrates Court, Abbey Road, Barrow in Furness, Cumbria, LA14 5QX</t>
+  </si>
+  <si>
+    <t>Blackpool Magistrates Court, Civic Centre, Chapel Street, Blackpool, Lancashire, FY1 5DQ</t>
+  </si>
+  <si>
+    <t>Piccadilly Exchange, 2 Piccadilly Plaza, Mosley Street, Manchester, M1 4AH</t>
+  </si>
+  <si>
+    <t>The Lowry Theatre Complex, Pier 8, Salford Quays, Salford, M50 3AZ</t>
+  </si>
+  <si>
+    <t>The Lowry</t>
+  </si>
+  <si>
+    <t>Leicester Hearing Centre, 5a New Walk, Leicester, LE1 6TE</t>
+  </si>
+  <si>
+    <t>Lincoln Magistrates Court, 358 High Street, Lincoln, LN5 7QA</t>
+  </si>
+  <si>
+    <t>Boston Court House, 55 Norfolk Street, Boston, PE21 6PE</t>
+  </si>
+  <si>
+    <t>Midlands West Employment Tribunal, Centre City Tower, 5-7 Hill Street, Birmingham, West Midlands, B5 4UU</t>
+  </si>
+  <si>
+    <t>Stoke-on-Trent Combined Court, Bethesda Street, Hanley, Stoke-on-Trent, T1 3BP</t>
+  </si>
+  <si>
+    <t>Telford Magistrates Court, Telford Square, Malinsgate, Telford, Shropshire, TF3 4HX</t>
+  </si>
+  <si>
+    <t>Reading Tribunal Hearing Centre 2nd Floor, 30-31 Friar Street, Reading, RG1 1DX</t>
+  </si>
+  <si>
+    <t>Amersham Law Courts King George V Road, Amersham, HP6 5AJ</t>
+  </si>
+  <si>
+    <t>Aylesbury Crown Court, Walton Street, Aylesbury, HP21 7FT</t>
+  </si>
+  <si>
+    <t>Huntingdon Law Courts Walden Rd, Huntingdon, PE29 3DW</t>
+  </si>
+  <si>
+    <t>Bedford County Court and Family Court, Shire Hall, 3 St Paul's Square, Bedford, MK40 1SQ</t>
+  </si>
+  <si>
+    <t>Cambridge County Court and Family Court, 197 East Road, Cambridge, CB1 1BA</t>
+  </si>
+  <si>
+    <t>Bury St Edmunds County Court and Family Court, Triton House, St Andrew's Street, North, Bury St. Edmunds, IP33 1TR</t>
+  </si>
+  <si>
+    <t>Norwich Magistrates' Court and Family Court, Bishopgate, Norwich, NR3 1UP</t>
+  </si>
+  <si>
+    <t>Peterborough</t>
+  </si>
+  <si>
+    <t>Peterborough nightingale Court Knights’ Chamber and Visitor Centre, Bishop’s, Palace, Peterborough Cathedral, Peterborough, PE1 1XZ</t>
+  </si>
+  <si>
+    <t>Campbeltown HC, Sheriff Court House, Castle Hill, Campbeltown, PA28 6AN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dumfries Sheriff Court </t>
+  </si>
+  <si>
+    <t>Dumfries HC, Sheriff Court House, Buccleuch Street, Dumfries, DG1 2AN</t>
+  </si>
+  <si>
+    <t>Oban HC, Sheriff Court House, Albany Street, Oban, PA34 4AL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oban Sheriff Court </t>
+  </si>
+  <si>
+    <t>Fort William SC, Sheriff Court House, High Street, Fort William, PH33 6EE</t>
+  </si>
+  <si>
+    <t>Kirkcudbright, Sheriff Court House, High Street, Kirkcudbright, DG6 4JW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lochmaddy Sheriff Court </t>
+  </si>
+  <si>
+    <t>Lochmaddy HC, Sheriff Court House, Lochmaddy, Isle of North Uist, HS6 5AE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portree Sheriff Court </t>
+  </si>
+  <si>
+    <t>Portree HC, Sheriff Court House, Somerled Square, Portree, IV51 9EH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stirling Sheriff Court </t>
+  </si>
+  <si>
+    <t>Stirling SC, Sheriff Court House, Viewfield Place, Stirling, FK8 1NH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stornoway Sheriff Court </t>
+  </si>
+  <si>
+    <t>Stornoway HC, Sheriff Court House, Lewis Street, Stornoway, Isle of Lewis, HS1 2JF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stranraer Sheriff Court </t>
+  </si>
+  <si>
+    <t>Stranraer HC, Sheriff Court House, Lewis Street, Stranraer, DG9 7AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lerwick </t>
+  </si>
+  <si>
+    <t>Lerwick Sheriff Court, King Erik Street, Lerwick, Shetland, ZE1 0HD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radio Room Shetland </t>
+  </si>
+  <si>
+    <t>Radio Room, Isleburgh Community Centre, Burgh Road, Shetland, ZE1 0EQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stornoway </t>
+  </si>
+  <si>
+    <t>Wick</t>
+  </si>
+  <si>
+    <t>Wick Sheriff Court House, Bridge Street, Wick, Caithness, KW1 4AJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inverness </t>
+  </si>
+  <si>
+    <t>Inverness Justice Centre, Longman Road, Inverness, IV1 1AH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kirkwall </t>
+  </si>
+  <si>
+    <t>Kirkwall Sheriff Court, Sheriff Court House, Watergate, Kirkwall, Orkney, KW15 1PD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campbeltown Sheriff Court </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fort William Sheriff Court </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kirkcudbright Sheriff Court </t>
+  </si>
+  <si>
+    <t>Hull Combined Court Centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cardiff SSCS </t>
+  </si>
+  <si>
+    <t>I J C</t>
+  </si>
+  <si>
+    <t>Longman Road, Inverness, IV1 1AH</t>
+  </si>
+  <si>
+    <t>Ground Floor, Endeavour House, 1 Greenmarket, Dundee, DD1 4QB</t>
+  </si>
+  <si>
+    <t>Hull Combined Court Centre, Lowgate, Hull, HU1 2EZ</t>
+  </si>
+  <si>
+    <t>Teesside Mags</t>
+  </si>
+  <si>
+    <t>Teesside Justice Centre, Victoria Square, Middlesbrough, Cleveland, TS1 2AS</t>
+  </si>
+  <si>
+    <t>2nd Floor, Radius House, 51 Clarendon Road, Watford, WD17 1HP</t>
+  </si>
+  <si>
+    <t>Tribunal Hearing Centre, 50 Carrington Street, Nottingham, NG1 7FG</t>
+  </si>
+  <si>
+    <t>Abergele Town Hall, Llanddulas Road, Abergele, Conwy, LL22 7BT</t>
+  </si>
+  <si>
+    <t>Leeds Westgate</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Aberystwyth Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Y Lanfa, Trefechan, Aberystwyth, SY23 1AS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Caernarfon Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Llanberis Road, Caernarfon, LL55 2DF</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cardiff Civil &amp; Family Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 2 Park Street, Cardiff, CF10 1ET</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cardiff Crown Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, The Law Courts, Cathays Park, Cardiff, CF10 3PG</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cardiff Magistrates’ Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Fitzalan Place, Cardiff, CF24 0RZ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Carmarthen County &amp; Family Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, The Hearing Centre, Hill House, Picton Terrace, Carmarthen, SA31 3BT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Haverfordwest County &amp; Family Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Penffynnon, Hawthorn Rise, Haverfordwest, SA61 2AX</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Llandudno Magistrates Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, The Court House, Conwy Road, Llandudno, LL30 1GA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Llanelli Law Courts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Town Hall Square, Llanelli, SA15 3AW</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mold Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Law Courts, Mold, CH7 1AE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Newport Immigration &amp; Asylum Tribunal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Columbus House, Langstone Business Park, Chepstow Road, Newport, NP18 2LX</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pontypridd County and Family Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, The Courthouse, Courthouse Street, Pontypridd, CF37 1JR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Port Talbot Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Harbourside Road, Port Talbot, SA13 1SB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Prestatyn Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Victoria Road, Prestatyn, LL19 7TE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Swansea Civil Justice Centre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Caravella House, Quay West, Quay Parade</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Swansea, SA1 1SP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Swansea Magistrates Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Grove Place, Swansea, SA1 5DB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wales Employment Tribunal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 3rd Floor, Cardiff Magistrates’ Court, Fitzalan Place, Cardiff, CF24 0RZ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Welshpool Magistrates Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Mansion House, 24 Severn Street, Welshpool, SY21 7UX</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wrexham County and Family Court</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, The Law Courts, Bodhyfryd, Wrexham, LL12 7BP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cardiff Social Security &amp; Child Support Tribunal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Eastgate House, 35-43 Newport Rd, Cardiff CF24 0AB</t>
+    </r>
+  </si>
+  <si>
+    <t>2nd Floor, West Gate , 6 Grace Street, Leeds, LS1 2RP</t>
+  </si>
+  <si>
+    <t>North Staffordshire Justice Centre</t>
+  </si>
+  <si>
+    <t>The Court House, Ryecroft, Newcastle-under-Lyme, ST5 2AA</t>
+  </si>
+  <si>
+    <t>London Tribunals Centre</t>
+  </si>
+  <si>
+    <t>7 Newgate Street, London, EC1A 7AZ</t>
+  </si>
+  <si>
+    <t>GTC</t>
+  </si>
+  <si>
+    <t>OET Scotland</t>
+  </si>
+  <si>
+    <t>OET 54-56 Melville Street, Edinburgh, EH3 7HF</t>
+  </si>
+  <si>
+    <t>Tribunal</t>
+  </si>
+  <si>
+    <t>Glasgow Tribunal Centre, 3 Atlantic Quay, 20 York Street, Glasgow, G2 8GT</t>
+  </si>
+  <si>
     <t>Victory House, 30-34 Kingsway, London, WC2B 6EX</t>
-  </si>
-  <si>
-    <t>London (Central), 4th Floor Fox Court, 30 Brooke Street, London, EC1N 7RS</t>
-  </si>
-  <si>
-    <t>East London Tribunals, 2nd Floor Import Building, 2 Clove Crescent, London,E 14 2BE</t>
-  </si>
-  <si>
-    <t>Newcastle CFCTC, Barras Bridge, Newcastle upon Tyne, Tyne &amp; Wear, NE1 8QF</t>
-  </si>
-  <si>
-    <t>Victoria Square, Middlesbrough, TS1 2AS</t>
-  </si>
-  <si>
-    <t>Earl Grey Way, North Shields, NE29 6AR</t>
-  </si>
-  <si>
-    <t>North Shields</t>
-  </si>
-  <si>
-    <t>Manchester Employment Tribunals, Alexandra House, 14-22 The Parsonage, Manchester, M3 2JA</t>
-  </si>
-  <si>
-    <t>Employment Tribunals, Third Floor, Civil &amp; Family Court, 35 Vernon Street, Liverpool, L2 2BX</t>
-  </si>
-  <si>
-    <t>Carlisle Combined Court, Courts of Justice, Earl Street, Carlisle, Cumbria, CA1 1DJ</t>
-  </si>
-  <si>
-    <t>Carlisle Magistrates Court, The Court House, Rickergate, Carlisle, CA3 8 QH</t>
-  </si>
-  <si>
-    <t>Barrow Magistrates Court, Abbey Road, Barrow in Furness, Cumbria, LA14 5QX</t>
-  </si>
-  <si>
-    <t>Blackpool Magistrates Court, Civic Centre, Chapel Street, Blackpool, Lancashire, FY1 5DQ</t>
-  </si>
-  <si>
-    <t>Piccadilly Exchange, 2 Piccadilly Plaza, Mosley Street, Manchester, M1 4AH</t>
-  </si>
-  <si>
-    <t>The Lowry Theatre Complex, Pier 8, Salford Quays, Salford, M50 3AZ</t>
-  </si>
-  <si>
-    <t>The Lowry</t>
-  </si>
-  <si>
-    <t>Leicester Hearing Centre, 5a New Walk, Leicester, LE1 6TE</t>
-  </si>
-  <si>
-    <t>Lincoln Magistrates Court, 358 High Street, Lincoln, LN5 7QA</t>
-  </si>
-  <si>
-    <t>Boston Court House, 55 Norfolk Street, Boston, PE21 6PE</t>
-  </si>
-  <si>
-    <t>Midlands West Employment Tribunal, Centre City Tower, 5-7 Hill Street, Birmingham, West Midlands, B5 4UU</t>
-  </si>
-  <si>
-    <t>Stoke-on-Trent Combined Court, Bethesda Street, Hanley, Stoke-on-Trent, T1 3BP</t>
-  </si>
-  <si>
-    <t>Telford Magistrates Court, Telford Square, Malinsgate, Telford, Shropshire, TF3 4HX</t>
-  </si>
-  <si>
-    <t>Reading Tribunal Hearing Centre 2nd Floor, 30-31 Friar Street, Reading, RG1 1DX</t>
-  </si>
-  <si>
-    <t>Amersham Law Courts King George V Road, Amersham, HP6 5AJ</t>
-  </si>
-  <si>
-    <t>Aylesbury Crown Court, Walton Street, Aylesbury, HP21 7FT</t>
-  </si>
-  <si>
-    <t>Huntingdon Law Courts Walden Rd, Huntingdon, PE29 3DW</t>
-  </si>
-  <si>
-    <t>Bedford County Court and Family Court, Shire Hall, 3 St Paul's Square, Bedford, MK40 1SQ</t>
-  </si>
-  <si>
-    <t>Cambridge County Court and Family Court, 197 East Road, Cambridge, CB1 1BA</t>
-  </si>
-  <si>
-    <t>Bury St Edmunds County Court and Family Court, Triton House, St Andrew's Street, North, Bury St. Edmunds, IP33 1TR</t>
-  </si>
-  <si>
-    <t>Norwich Magistrates' Court and Family Court, Bishopgate, Norwich, NR3 1UP</t>
-  </si>
-  <si>
-    <t>Peterborough</t>
-  </si>
-  <si>
-    <t>Peterborough nightingale Court Knights’ Chamber and Visitor Centre, Bishop’s, Palace, Peterborough Cathedral, Peterborough, PE1 1XZ</t>
-  </si>
-  <si>
-    <t>Campbeltown HC, Sheriff Court House, Castle Hill, Campbeltown, PA28 6AN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dumfries Sheriff Court </t>
-  </si>
-  <si>
-    <t>Dumfries HC, Sheriff Court House, Buccleuch Street, Dumfries, DG1 2AN</t>
-  </si>
-  <si>
-    <t>Oban HC, Sheriff Court House, Albany Street, Oban, PA34 4AL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oban Sheriff Court </t>
-  </si>
-  <si>
-    <t>Fort William SC, Sheriff Court House, High Street, Fort William, PH33 6EE</t>
-  </si>
-  <si>
-    <t>Kirkcudbright, Sheriff Court House, High Street, Kirkcudbright, DG6 4JW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lochmaddy Sheriff Court </t>
-  </si>
-  <si>
-    <t>Lochmaddy HC, Sheriff Court House, Lochmaddy, Isle of North Uist, HS6 5AE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portree Sheriff Court </t>
-  </si>
-  <si>
-    <t>Portree HC, Sheriff Court House, Somerled Square, Portree, IV51 9EH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stirling Sheriff Court </t>
-  </si>
-  <si>
-    <t>Stirling SC, Sheriff Court House, Viewfield Place, Stirling, FK8 1NH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stornoway Sheriff Court </t>
-  </si>
-  <si>
-    <t>Stornoway HC, Sheriff Court House, Lewis Street, Stornoway, Isle of Lewis, HS1 2JF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stranraer Sheriff Court </t>
-  </si>
-  <si>
-    <t>Stranraer HC, Sheriff Court House, Lewis Street, Stranraer, DG9 7AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lerwick </t>
-  </si>
-  <si>
-    <t>Lerwick Sheriff Court, King Erik Street, Lerwick, Shetland, ZE1 0HD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Radio Room Shetland </t>
-  </si>
-  <si>
-    <t>Radio Room, Isleburgh Community Centre, Burgh Road, Shetland, ZE1 0EQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stornoway </t>
-  </si>
-  <si>
-    <t>Wick</t>
-  </si>
-  <si>
-    <t>Wick Sheriff Court House, Bridge Street, Wick, Caithness, KW1 4AJ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inverness </t>
-  </si>
-  <si>
-    <t>Inverness Justice Centre, Longman Road, Inverness, IV1 1AH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kirkwall </t>
-  </si>
-  <si>
-    <t>Kirkwall Sheriff Court, Sheriff Court House, Watergate, Kirkwall, Orkney, KW15 1PD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campbeltown Sheriff Court </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fort William Sheriff Court </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kirkcudbright Sheriff Court </t>
-  </si>
-  <si>
-    <t>Hull Combined Court Centre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cardiff SSCS </t>
-  </si>
-  <si>
-    <t>I J C</t>
-  </si>
-  <si>
-    <t>Longman Road, Inverness, IV1 1AH</t>
-  </si>
-  <si>
-    <t>Ground Floor, Endeavour House, 1 Greenmarket, Dundee, DD1 4QB</t>
-  </si>
-  <si>
-    <t>Hull Combined Court Centre, Lowgate, Hull, HU1 2EZ</t>
-  </si>
-  <si>
-    <t>Teesside Mags</t>
-  </si>
-  <si>
-    <t>Teesside Justice Centre, Victoria Square, Middlesbrough, Cleveland, TS1 2AS</t>
-  </si>
-  <si>
-    <t>2nd Floor, Radius House, 51 Clarendon Road, Watford, WD17 1HP</t>
-  </si>
-  <si>
-    <t>Tribunal Hearing Centre, 50 Carrington Street, Nottingham, NG1 7FG</t>
-  </si>
-  <si>
-    <t>Abergele Town Hall, Llanddulas Road, Abergele, Conwy, LL22 7BT</t>
-  </si>
-  <si>
-    <t>Leeds Westgate</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Aberystwyth Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Y Lanfa, Trefechan, Aberystwyth, SY23 1AS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Caernarfon Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Llanberis Road, Caernarfon, LL55 2DF</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cardiff Civil &amp; Family Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 2 Park Street, Cardiff, CF10 1ET</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cardiff Crown Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, The Law Courts, Cathays Park, Cardiff, CF10 3PG</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cardiff Magistrates’ Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Fitzalan Place, Cardiff, CF24 0RZ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Carmarthen County &amp; Family Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, The Hearing Centre, Hill House, Picton Terrace, Carmarthen, SA31 3BT</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Haverfordwest County &amp; Family Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Penffynnon, Hawthorn Rise, Haverfordwest, SA61 2AX</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Llandudno Magistrates Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, The Court House, Conwy Road, Llandudno, LL30 1GA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Llanelli Law Courts</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Town Hall Square, Llanelli, SA15 3AW</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mold Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Law Courts, Mold, CH7 1AE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Newport Immigration &amp; Asylum Tribunal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Columbus House, Langstone Business Park, Chepstow Road, Newport, NP18 2LX</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Pontypridd County and Family Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, The Courthouse, Courthouse Street, Pontypridd, CF37 1JR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Port Talbot Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Harbourside Road, Port Talbot, SA13 1SB</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Prestatyn Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Victoria Road, Prestatyn, LL19 7TE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Swansea Civil Justice Centre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Caravella House, Quay West, Quay Parade</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Swansea, SA1 1SP</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Swansea Magistrates Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Grove Place, Swansea, SA1 5DB</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wales Employment Tribunal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 3rd Floor, Cardiff Magistrates’ Court, Fitzalan Place, Cardiff, CF24 0RZ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Welshpool Magistrates Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Mansion House, 24 Severn Street, Welshpool, SY21 7UX</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wrexham County and Family Court</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, The Law Courts, Bodhyfryd, Wrexham, LL12 7BP</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cardiff Social Security &amp; Child Support Tribunal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Eastgate House, 35-43 Newport Rd, Cardiff CF24 0AB</t>
-    </r>
-  </si>
-  <si>
-    <t>2nd Floor, West Gate , 6 Grace Street, Leeds, LS1 2RP</t>
-  </si>
-  <si>
-    <t>North Staffordshire Justice Centre</t>
-  </si>
-  <si>
-    <t>The Court House, Ryecroft, Newcastle-under-Lyme, ST5 2AA</t>
-  </si>
-  <si>
-    <t>London Tribunals Centre</t>
-  </si>
-  <si>
-    <t>7 Newgate Street, London, EC1A 7AZ</t>
-  </si>
-  <si>
-    <t>GTC</t>
-  </si>
-  <si>
-    <t>OET Scotland</t>
-  </si>
-  <si>
-    <t>OET 54-56 Melville Street, Edinburgh, EH3 7HF</t>
-  </si>
-  <si>
-    <t>Tribunal</t>
-  </si>
-  <si>
-    <t>Glasgow Tribunal Centre, 3 Atlantic Quay, 20 York Street, Glasgow, G2 8GT</t>
   </si>
 </sst>
 </file>
@@ -2142,18 +2142,18 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>231</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2174,10 +2174,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2190,138 +2190,138 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>254</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>247</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>237</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>249</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>243</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>245</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -2363,7 +2363,7 @@
         <v>104</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2379,7 +2379,7 @@
         <v>106</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2411,7 +2411,7 @@
         <v>110</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2427,7 +2427,7 @@
         <v>112</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2435,7 +2435,7 @@
         <v>113</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2459,7 +2459,7 @@
         <v>116</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -2491,7 +2491,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2579,7 +2579,7 @@
         <v>131</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -2635,7 +2635,7 @@
         <v>138</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -2651,7 +2651,7 @@
         <v>140</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -2683,7 +2683,7 @@
         <v>144</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -2723,7 +2723,7 @@
         <v>149</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -2739,7 +2739,7 @@
         <v>151</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -2747,7 +2747,7 @@
         <v>152</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -2755,7 +2755,7 @@
         <v>153</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -2795,7 +2795,7 @@
         <v>158</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -2811,7 +2811,7 @@
         <v>160</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -2843,7 +2843,7 @@
         <v>164</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -2851,7 +2851,7 @@
         <v>165</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -2867,7 +2867,7 @@
         <v>167</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -2880,10 +2880,10 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2915,7 +2915,7 @@
         <v>169</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2923,7 +2923,7 @@
         <v>170</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2931,7 +2931,7 @@
         <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2947,7 +2947,7 @@
         <v>89</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2955,7 +2955,7 @@
         <v>90</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2963,7 +2963,7 @@
         <v>172</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2987,7 +2987,7 @@
         <v>174</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2995,7 +2995,7 @@
         <v>175</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3011,15 +3011,15 @@
         <v>177</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>228</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3071,10 +3071,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3111,10 +3111,10 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3153,7 +3153,7 @@
         <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3161,15 +3161,15 @@
         <v>51</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>296</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3216,7 +3216,7 @@
         <v>54</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3310,7 +3310,7 @@
         <v>60</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3318,7 +3318,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3334,7 +3334,7 @@
         <v>63</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3342,7 +3342,7 @@
         <v>64</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3382,7 +3382,7 @@
         <v>69</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3390,7 +3390,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3398,7 +3398,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3427,10 +3427,10 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -3469,7 +3469,7 @@
         <v>75</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3493,7 +3493,7 @@
         <v>78</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3501,7 +3501,7 @@
         <v>79</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3525,7 +3525,7 @@
         <v>81</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3604,7 +3604,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3641,10 +3641,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3660,7 +3660,7 @@
         <v>93</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3668,7 +3668,7 @@
         <v>94</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3739,7 +3739,7 @@
         <v>100</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3747,7 +3747,7 @@
         <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3768,18 +3768,18 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -3788,21 +3788,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E98ADB2028FC4F43824F86666CC83903" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff47f26d8558bca2ac2c896a7e751c25">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="bc19a69a-bda7-4614-8881-f2ac618cff8e" xmlns:ns4="02128cc3-8226-4d54-9246-100bb62c9520" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="63ef4ea587d9ab0193671c85d2373b1f" ns3:_="" ns4:_="">
     <xsd:import namespace="bc19a69a-bda7-4614-8881-f2ac618cff8e"/>
@@ -4019,24 +4004,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E254D28-D3D4-49BF-9139-FF4FDEF467DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E21D230-F0FF-46F1-8C9B-DF853E5491B6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00A2FE85-4E03-4320-929A-8E66617AF346}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4053,4 +4036,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E254D28-D3D4-49BF-9139-FF4FDEF467DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E21D230-F0FF-46F1-8C9B-DF853E5491B6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>